<commit_message>
Update SLURM files with email message, remove young-age targets with few cases
</commit_message>
<xml_diff>
--- a/data/colorectal/targets.xlsx
+++ b/data/colorectal/targets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/selinapi/Repositories/tutorial_cancer_modeling_des/data/colorectal/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5512562-BEB3-2741-83D9-99624FFFB55E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD470353-B6B9-144E-9706-D4BA2E94BD37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17740" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17740" activeTab="1" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
   </bookViews>
   <sheets>
     <sheet name="targets" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="37">
   <si>
     <t>target_names</t>
   </si>
@@ -539,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B407C086-A524-D44D-8D0D-4CA59B33056E}">
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25.33203125" style="1" customWidth="1"/>
@@ -1261,33 +1261,33 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="str">
-        <f t="shared" ref="A20:A40" si="4">""&amp;B20&amp;"_"&amp;E20</f>
-        <v>prevalence_preclin_10</v>
+        <f t="shared" ref="A20:A36" si="4">""&amp;B20&amp;"_"&amp;E20</f>
+        <v>prevalence_preclin_35</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C20" s="2">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="D20" s="2">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E20" s="1">
-        <f t="shared" ref="E20:E28" si="5">FLOOR(AVERAGE(C20,D20), 1)</f>
-        <v>10</v>
+        <f t="shared" ref="E20:E26" si="5">FLOOR(AVERAGE(C20,D20), 1)</f>
+        <v>35</v>
       </c>
       <c r="F20" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A20,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>0</v>
+        <v>2.9069767441860465E-3</v>
       </c>
       <c r="G20" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A20,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>0</v>
+        <v>5.1333721812770253E-4</v>
       </c>
       <c r="H20" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A20,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>2.3199436155137984E-3</v>
+        <v>1.6280114719714151E-2</v>
       </c>
       <c r="I20" s="1" t="s">
         <v>8</v>
@@ -1302,32 +1302,32 @@
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>prevalence_preclin_25</v>
+        <v>prevalence_preclin_45</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C21" s="2">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="D21" s="2">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="E21" s="1">
         <f t="shared" si="5"/>
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="F21" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A21,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>0</v>
+        <v>5.4844606946983544E-3</v>
       </c>
       <c r="G21" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A21,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>0</v>
+        <v>1.8669281252303872E-3</v>
       </c>
       <c r="H21" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A21,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>2.1125318976251823E-2</v>
+        <v>1.5999299376533674E-2</v>
       </c>
       <c r="I21" s="1" t="s">
         <v>8</v>
@@ -1342,32 +1342,32 @@
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>prevalence_preclin_35</v>
+        <v>prevalence_preclin_55</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C22" s="2">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D22" s="2">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="E22" s="1">
         <f t="shared" si="5"/>
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="F22" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A22,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>2.9069767441860465E-3</v>
+        <v>6.7024128686327079E-3</v>
       </c>
       <c r="G22" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A22,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>5.1333721812770253E-4</v>
+        <v>2.8661685080304854E-3</v>
       </c>
       <c r="H22" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A22,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>1.6280114719714151E-2</v>
+        <v>1.5593011973218367E-2</v>
       </c>
       <c r="I22" s="1" t="s">
         <v>8</v>
@@ -1382,32 +1382,32 @@
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>prevalence_preclin_45</v>
+        <v>prevalence_preclin_65</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C23" s="2">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="D23" s="2">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E23" s="1">
         <f t="shared" si="5"/>
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="F23" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>5.4844606946983544E-3</v>
+        <v>1.5682656826568265E-2</v>
       </c>
       <c r="G23" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>1.8669281252303872E-3</v>
+        <v>9.8142486381670446E-3</v>
       </c>
       <c r="H23" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>1.5999299376533674E-2</v>
+        <v>2.4971572874571808E-2</v>
       </c>
       <c r="I23" s="1" t="s">
         <v>8</v>
@@ -1422,32 +1422,32 @@
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>prevalence_preclin_55</v>
+        <v>prevalence_preclin_75</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C24" s="2">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="D24" s="2">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="E24" s="1">
         <f t="shared" si="5"/>
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="F24" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>6.7024128686327079E-3</v>
+        <v>1.8207282913165267E-2</v>
       </c>
       <c r="G24" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>2.8661685080304854E-3</v>
+        <v>1.2455064037696518E-2</v>
       </c>
       <c r="H24" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>1.5593011973218367E-2</v>
+        <v>2.6544685883420276E-2</v>
       </c>
       <c r="I24" s="1" t="s">
         <v>8</v>
@@ -1462,32 +1462,32 @@
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>prevalence_preclin_65</v>
+        <v>prevalence_preclin_85</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C25" s="2">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="D25" s="2">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="E25" s="1">
         <f t="shared" si="5"/>
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="F25" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>1.5682656826568265E-2</v>
+        <v>2.5930101465614429E-2</v>
       </c>
       <c r="G25" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>9.8142486381670446E-3</v>
+        <v>1.7339774526665963E-2</v>
       </c>
       <c r="H25" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>2.4971572874571808E-2</v>
+        <v>3.8608967336644713E-2</v>
       </c>
       <c r="I25" s="1" t="s">
         <v>8</v>
@@ -1502,32 +1502,32 @@
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>prevalence_preclin_75</v>
+        <v>prevalence_preclin_95</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C26" s="2">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="D26" s="2">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="E26" s="1">
         <f t="shared" si="5"/>
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="F26" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A26,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>1.8207282913165267E-2</v>
+        <v>1.3333333333333334E-2</v>
       </c>
       <c r="G26" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A26,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>1.2455064037696518E-2</v>
+        <v>3.6641291512270503E-3</v>
       </c>
       <c r="H26" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A26,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>2.6544685883420276E-2</v>
+        <v>4.7306908700367495E-2</v>
       </c>
       <c r="I26" s="1" t="s">
         <v>8</v>
@@ -1542,32 +1542,30 @@
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>prevalence_preclin_85</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C27" s="2">
-        <v>80</v>
-      </c>
-      <c r="D27" s="2">
-        <v>90</v>
+        <v>incidence_clin_35</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C27" s="1">
+        <v>30</v>
+      </c>
+      <c r="D27" s="1">
+        <f>C28</f>
+        <v>40</v>
       </c>
       <c r="E27" s="1">
-        <f t="shared" si="5"/>
-        <v>85</v>
-      </c>
-      <c r="F27" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A27,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>2.5930101465614429E-2</v>
-      </c>
-      <c r="G27" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A27,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>1.7339774526665963E-2</v>
-      </c>
-      <c r="H27" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A27,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>3.8608967336644713E-2</v>
+        <f t="shared" ref="E27" si="6">FLOOR(AVERAGE(C27,D27), 1)</f>
+        <v>35</v>
+      </c>
+      <c r="F27" s="1">
+        <v>4.1520000000000001</v>
+      </c>
+      <c r="G27" s="1">
+        <v>3.6070000000000002</v>
+      </c>
+      <c r="H27" s="1">
+        <v>4.7519999999999998</v>
       </c>
       <c r="I27" s="1" t="s">
         <v>8</v>
@@ -1576,38 +1574,36 @@
         <v>13</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>prevalence_preclin_95</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C28" s="2">
-        <v>90</v>
-      </c>
-      <c r="D28" s="2">
-        <v>100</v>
+        <v>incidence_clin_45</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C28" s="1">
+        <v>40</v>
+      </c>
+      <c r="D28" s="1">
+        <f t="shared" ref="D28:D31" si="7">C29</f>
+        <v>50</v>
       </c>
       <c r="E28" s="1">
-        <f t="shared" si="5"/>
-        <v>95</v>
-      </c>
-      <c r="F28" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A28,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>1.3333333333333334E-2</v>
-      </c>
-      <c r="G28" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A28,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>3.6641291512270503E-3</v>
-      </c>
-      <c r="H28" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A28,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>4.7306908700367495E-2</v>
+        <f t="shared" ref="E28:E32" si="8">FLOOR(AVERAGE(C28,D28), 1)</f>
+        <v>45</v>
+      </c>
+      <c r="F28" s="1">
+        <v>20.667999999999999</v>
+      </c>
+      <c r="G28" s="1">
+        <v>19.263999999999999</v>
+      </c>
+      <c r="H28" s="1">
+        <v>22.140999999999998</v>
       </c>
       <c r="I28" s="1" t="s">
         <v>8</v>
@@ -1616,36 +1612,36 @@
         <v>13</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>incidence_clin_10</v>
+        <v>incidence_clin_55</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C29" s="1">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="D29" s="1">
-        <f>C30</f>
-        <v>20</v>
+        <f t="shared" si="7"/>
+        <v>60</v>
       </c>
       <c r="E29" s="1">
-        <f t="shared" ref="E29" si="6">FLOOR(AVERAGE(C29,D29), 1)</f>
-        <v>10</v>
+        <f t="shared" si="8"/>
+        <v>55</v>
       </c>
       <c r="F29" s="1">
-        <v>0</v>
+        <v>69.337999999999994</v>
       </c>
       <c r="G29" s="1">
-        <v>0</v>
+        <v>66.747</v>
       </c>
       <c r="H29" s="1">
-        <v>2.1999999999999999E-2</v>
+        <v>71.998999999999995</v>
       </c>
       <c r="I29" s="1" t="s">
         <v>8</v>
@@ -1660,30 +1656,30 @@
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>incidence_clin_25</v>
+        <v>incidence_clin_65</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C30" s="1">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="D30" s="1">
-        <f>C31</f>
-        <v>30</v>
+        <f t="shared" si="7"/>
+        <v>70</v>
       </c>
       <c r="E30" s="1">
-        <f t="shared" ref="E30" si="7">FLOOR(AVERAGE(C30,D30), 1)</f>
-        <v>25</v>
+        <f t="shared" si="8"/>
+        <v>65</v>
       </c>
       <c r="F30" s="1">
-        <v>0.81499999999999995</v>
+        <v>166.136</v>
       </c>
       <c r="G30" s="1">
-        <v>0.61499999999999999</v>
+        <v>161.41399999999999</v>
       </c>
       <c r="H30" s="1">
-        <v>1.0549999999999999</v>
+        <v>170.952</v>
       </c>
       <c r="I30" s="1" t="s">
         <v>8</v>
@@ -1698,30 +1694,30 @@
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>incidence_clin_35</v>
+        <v>incidence_clin_75</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C31" s="1">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="D31" s="1">
-        <f>C32</f>
-        <v>40</v>
+        <f t="shared" si="7"/>
+        <v>80</v>
       </c>
       <c r="E31" s="1">
-        <f t="shared" ref="E31" si="8">FLOOR(AVERAGE(C31,D31), 1)</f>
-        <v>35</v>
+        <f t="shared" si="8"/>
+        <v>75</v>
       </c>
       <c r="F31" s="1">
-        <v>4.1520000000000001</v>
+        <v>309.19900000000001</v>
       </c>
       <c r="G31" s="1">
-        <v>3.6070000000000002</v>
+        <v>300.73399999999998</v>
       </c>
       <c r="H31" s="1">
-        <v>4.7519999999999998</v>
+        <v>317.83</v>
       </c>
       <c r="I31" s="1" t="s">
         <v>8</v>
@@ -1736,30 +1732,29 @@
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>incidence_clin_45</v>
+        <v>incidence_clin_90</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C32" s="1">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="D32" s="1">
-        <f t="shared" ref="D32:D35" si="9">C33</f>
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="E32" s="1">
-        <f t="shared" ref="E32:E36" si="10">FLOOR(AVERAGE(C32,D32), 1)</f>
-        <v>45</v>
+        <f t="shared" si="8"/>
+        <v>90</v>
       </c>
       <c r="F32" s="1">
-        <v>20.667999999999999</v>
+        <v>428.28899999999999</v>
       </c>
       <c r="G32" s="1">
-        <v>19.263999999999999</v>
+        <v>413.87099999999998</v>
       </c>
       <c r="H32" s="1">
-        <v>22.140999999999998</v>
+        <v>443.053</v>
       </c>
       <c r="I32" s="1" t="s">
         <v>8</v>
@@ -1774,30 +1769,25 @@
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>incidence_clin_55</v>
+        <v>stage_distr_1</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C33" s="1">
-        <v>50</v>
-      </c>
-      <c r="D33" s="1">
-        <f t="shared" si="9"/>
-        <v>60</v>
+        <v>17</v>
       </c>
       <c r="E33" s="1">
-        <f t="shared" si="10"/>
-        <v>55</v>
-      </c>
-      <c r="F33" s="1">
-        <v>69.337999999999994</v>
-      </c>
-      <c r="G33" s="1">
-        <v>66.747</v>
-      </c>
-      <c r="H33" s="1">
-        <v>71.998999999999995</v>
+        <v>1</v>
+      </c>
+      <c r="F33" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A33,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <v>0.18080563434143854</v>
+      </c>
+      <c r="G33" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A33,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
+        <v>0.17781418443524724</v>
+      </c>
+      <c r="H33" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A33,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
+        <v>0.18383615805371881</v>
       </c>
       <c r="I33" s="1" t="s">
         <v>8</v>
@@ -1812,30 +1802,25 @@
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>incidence_clin_65</v>
+        <v>stage_distr_2</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C34" s="1">
-        <v>60</v>
-      </c>
-      <c r="D34" s="1">
-        <f t="shared" si="9"/>
-        <v>70</v>
+        <v>17</v>
       </c>
       <c r="E34" s="1">
-        <f t="shared" si="10"/>
-        <v>65</v>
-      </c>
-      <c r="F34" s="1">
-        <v>166.136</v>
-      </c>
-      <c r="G34" s="1">
-        <v>161.41399999999999</v>
-      </c>
-      <c r="H34" s="1">
-        <v>170.952</v>
+        <v>2</v>
+      </c>
+      <c r="F34" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A34,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <v>0.33584562924248701</v>
+      </c>
+      <c r="G34" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A34,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
+        <v>0.33216074653492256</v>
+      </c>
+      <c r="H34" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A34,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
+        <v>0.33955060671594262</v>
       </c>
       <c r="I34" s="1" t="s">
         <v>8</v>
@@ -1850,30 +1835,25 @@
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>incidence_clin_75</v>
+        <v>stage_distr_3</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C35" s="1">
-        <v>70</v>
-      </c>
-      <c r="D35" s="1">
-        <f t="shared" si="9"/>
-        <v>80</v>
+        <v>17</v>
       </c>
       <c r="E35" s="1">
-        <f t="shared" si="10"/>
-        <v>75</v>
-      </c>
-      <c r="F35" s="1">
-        <v>309.19900000000001</v>
-      </c>
-      <c r="G35" s="1">
-        <v>300.73399999999998</v>
-      </c>
-      <c r="H35" s="1">
-        <v>317.83</v>
+        <v>3</v>
+      </c>
+      <c r="F35" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A35,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <v>0.24546671340705567</v>
+      </c>
+      <c r="G35" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A35,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
+        <v>0.24211531360934294</v>
+      </c>
+      <c r="H35" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A35,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
+        <v>0.24884927160025891</v>
       </c>
       <c r="I35" s="1" t="s">
         <v>8</v>
@@ -1888,29 +1868,25 @@
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>incidence_clin_90</v>
+        <v>stage_distr_4</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C36" s="1">
-        <v>80</v>
-      </c>
-      <c r="D36" s="1">
-        <v>100</v>
+        <v>17</v>
       </c>
       <c r="E36" s="1">
-        <f t="shared" si="10"/>
-        <v>90</v>
-      </c>
-      <c r="F36" s="1">
-        <v>428.28899999999999</v>
-      </c>
-      <c r="G36" s="1">
-        <v>413.87099999999998</v>
-      </c>
-      <c r="H36" s="1">
-        <v>443.053</v>
+        <v>4</v>
+      </c>
+      <c r="F36" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A36,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <v>0.23788202300901878</v>
+      </c>
+      <c r="G36" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A36,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
+        <v>0.23456689332002215</v>
+      </c>
+      <c r="H36" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A36,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
+        <v>0.24122923956453721</v>
       </c>
       <c r="I36" s="1" t="s">
         <v>8</v>
@@ -1919,138 +1895,6 @@
         <v>13</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A37" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>stage_distr_1</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E37" s="1">
-        <v>1</v>
-      </c>
-      <c r="F37" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A37,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>0.18080563434143854</v>
-      </c>
-      <c r="G37" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A37,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>0.17781418443524724</v>
-      </c>
-      <c r="H37" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A37,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>0.18383615805371881</v>
-      </c>
-      <c r="I37" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J37" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K37" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A38" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>stage_distr_2</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E38" s="1">
-        <v>2</v>
-      </c>
-      <c r="F38" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A38,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>0.33584562924248701</v>
-      </c>
-      <c r="G38" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A38,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>0.33216074653492256</v>
-      </c>
-      <c r="H38" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A38,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>0.33955060671594262</v>
-      </c>
-      <c r="I38" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J38" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K38" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A39" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>stage_distr_3</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E39" s="1">
-        <v>3</v>
-      </c>
-      <c r="F39" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A39,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>0.24546671340705567</v>
-      </c>
-      <c r="G39" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A39,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>0.24211531360934294</v>
-      </c>
-      <c r="H39" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A39,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>0.24884927160025891</v>
-      </c>
-      <c r="I39" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J39" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K39" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A40" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>stage_distr_4</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E40" s="1">
-        <v>4</v>
-      </c>
-      <c r="F40" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A40,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>0.23788202300901878</v>
-      </c>
-      <c r="G40" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A40,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>0.23456689332002215</v>
-      </c>
-      <c r="H40" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A40,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>0.24122923956453721</v>
-      </c>
-      <c r="I40" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J40" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K40" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -2062,10 +1906,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79E831A2-898F-7F45-AC2C-D0D6D35A5E8A}">
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="1" width="32.1640625" style="1" customWidth="1"/>
+    <col min="2" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
@@ -2135,425 +1980,409 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="str">
-        <f>"prevalence_preclin_"&amp;E7</f>
-        <v>prevalence_preclin_10</v>
+        <f t="shared" ref="A7" si="0">"prevalence_preclin_"&amp;E7</f>
+        <v>prevalence_preclin_35</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C7" s="1">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="D7" s="1">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E7" s="1">
-        <f t="shared" ref="E7:E15" si="0">FLOOR(AVERAGE(C7,D7), 1)</f>
-        <v>10</v>
+        <f t="shared" ref="E7:E13" si="1">FLOOR(AVERAGE(C7,D7), 1)</f>
+        <v>35</v>
       </c>
       <c r="G7" s="1">
-        <v>1652</v>
+        <v>344</v>
       </c>
       <c r="H7" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7" s="1">
-        <f>H7/G7</f>
-        <v>0</v>
+        <f t="shared" ref="I7:I13" si="2">H7/G7</f>
+        <v>2.9069767441860465E-3</v>
       </c>
       <c r="J7" s="1">
-        <f t="shared" ref="J7:J15" si="1">$B$4^2/G7</f>
-        <v>2.3253382691853048E-3</v>
+        <f t="shared" ref="J7:J13" si="3">$B$4^2/G7</f>
+        <v>1.1167031455506174E-2</v>
       </c>
       <c r="K7" s="1">
-        <f t="shared" ref="K7:K15" si="2">(I7+J7/2)/(J7+1)-$B$4/(J7+1)*SQRT(I7*(1-I7)/G7+J7/(4*G7))</f>
-        <v>0</v>
+        <f t="shared" ref="K7:K13" si="4">(I7+J7/2)/(J7+1)-$B$4/(J7+1)*SQRT(I7*(1-I7)/G7+J7/(4*G7))</f>
+        <v>5.1333721812770253E-4</v>
       </c>
       <c r="L7" s="1">
-        <f t="shared" ref="L7:L15" si="3">(I7+J7/2)/(J7+1)+$B$4/(J7+1)*SQRT(I7*(1-I7)/G7+J7/(4*G7))</f>
-        <v>2.3199436155137984E-3</v>
+        <f t="shared" ref="L7:L13" si="5">(I7+J7/2)/(J7+1)+$B$4/(J7+1)*SQRT(I7*(1-I7)/G7+J7/(4*G7))</f>
+        <v>1.6280114719714151E-2</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="str">
-        <f t="shared" ref="A8:A9" si="4">"prevalence_preclin_"&amp;E8</f>
-        <v>prevalence_preclin_25</v>
+        <f t="shared" ref="A8:A13" si="6">"prevalence_preclin_"&amp;E8</f>
+        <v>prevalence_preclin_45</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C8" s="1">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="D8" s="1">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="E8" s="1">
-        <f t="shared" si="0"/>
-        <v>25</v>
+        <f t="shared" si="1"/>
+        <v>45</v>
       </c>
       <c r="G8" s="1">
-        <v>178</v>
+        <v>547</v>
       </c>
       <c r="H8" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I8" s="1">
-        <f t="shared" ref="I8:I15" si="5">H8/G8</f>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>5.4844606946983544E-3</v>
       </c>
       <c r="J8" s="1">
-        <f t="shared" si="1"/>
-        <v>2.1581229329742269E-2</v>
+        <f t="shared" si="3"/>
+        <v>7.0227766374664049E-3</v>
       </c>
       <c r="K8" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>1.8669281252303872E-3</v>
       </c>
       <c r="L8" s="1">
-        <f t="shared" si="3"/>
-        <v>2.1125318976251823E-2</v>
+        <f t="shared" si="5"/>
+        <v>1.5999299376533674E-2</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>prevalence_preclin_35</v>
+        <f t="shared" si="6"/>
+        <v>prevalence_preclin_55</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C9" s="1">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D9" s="1">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="E9" s="1">
-        <f t="shared" si="0"/>
-        <v>35</v>
+        <f t="shared" si="1"/>
+        <v>55</v>
       </c>
       <c r="G9" s="1">
-        <v>344</v>
+        <v>746</v>
       </c>
       <c r="H9" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I9" s="1">
+        <f t="shared" si="2"/>
+        <v>6.7024128686327079E-3</v>
+      </c>
+      <c r="J9" s="1">
+        <f t="shared" si="3"/>
+        <v>5.1494086068285842E-3</v>
+      </c>
+      <c r="K9" s="1">
+        <f t="shared" si="4"/>
+        <v>2.8661685080304854E-3</v>
+      </c>
+      <c r="L9" s="1">
         <f t="shared" si="5"/>
-        <v>2.9069767441860465E-3</v>
-      </c>
-      <c r="J9" s="1">
-        <f t="shared" si="1"/>
-        <v>1.1167031455506174E-2</v>
-      </c>
-      <c r="K9" s="1">
-        <f t="shared" si="2"/>
-        <v>5.1333721812770253E-4</v>
-      </c>
-      <c r="L9" s="1">
-        <f t="shared" si="3"/>
-        <v>1.6280114719714151E-2</v>
+        <v>1.5593011973218367E-2</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="str">
-        <f t="shared" ref="A10:A15" si="6">"prevalence_preclin_"&amp;E10</f>
-        <v>prevalence_preclin_45</v>
+        <f t="shared" si="6"/>
+        <v>prevalence_preclin_65</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="1">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="D10" s="1">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E10" s="1">
-        <f t="shared" si="0"/>
-        <v>45</v>
+        <f t="shared" si="1"/>
+        <v>65</v>
       </c>
       <c r="G10" s="1">
-        <v>547</v>
+        <v>1084</v>
       </c>
       <c r="H10" s="1">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="I10" s="1">
+        <f t="shared" si="2"/>
+        <v>1.5682656826568265E-2</v>
+      </c>
+      <c r="J10" s="1">
+        <f t="shared" si="3"/>
+        <v>3.543781199902328E-3</v>
+      </c>
+      <c r="K10" s="1">
+        <f t="shared" si="4"/>
+        <v>9.8142486381670446E-3</v>
+      </c>
+      <c r="L10" s="1">
         <f t="shared" si="5"/>
-        <v>5.4844606946983544E-3</v>
-      </c>
-      <c r="J10" s="1">
-        <f t="shared" si="1"/>
-        <v>7.0227766374664049E-3</v>
-      </c>
-      <c r="K10" s="1">
-        <f t="shared" si="2"/>
-        <v>1.8669281252303872E-3</v>
-      </c>
-      <c r="L10" s="1">
-        <f t="shared" si="3"/>
-        <v>1.5999299376533674E-2</v>
+        <v>2.4971572874571808E-2</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="str">
         <f t="shared" si="6"/>
-        <v>prevalence_preclin_55</v>
+        <v>prevalence_preclin_75</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C11" s="1">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="D11" s="1">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="E11" s="1">
-        <f t="shared" si="0"/>
-        <v>55</v>
+        <f t="shared" si="1"/>
+        <v>75</v>
       </c>
       <c r="G11" s="1">
-        <v>746</v>
+        <v>1428</v>
       </c>
       <c r="H11" s="1">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="I11" s="1">
+        <f t="shared" si="2"/>
+        <v>1.8207282913165267E-2</v>
+      </c>
+      <c r="J11" s="1">
+        <f t="shared" si="3"/>
+        <v>2.690097213371235E-3</v>
+      </c>
+      <c r="K11" s="1">
+        <f t="shared" si="4"/>
+        <v>1.2455064037696518E-2</v>
+      </c>
+      <c r="L11" s="1">
         <f t="shared" si="5"/>
-        <v>6.7024128686327079E-3</v>
-      </c>
-      <c r="J11" s="1">
-        <f t="shared" si="1"/>
-        <v>5.1494086068285842E-3</v>
-      </c>
-      <c r="K11" s="1">
-        <f t="shared" si="2"/>
-        <v>2.8661685080304854E-3</v>
-      </c>
-      <c r="L11" s="1">
-        <f t="shared" si="3"/>
-        <v>1.5593011973218367E-2</v>
+        <v>2.6544685883420276E-2</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="str">
         <f t="shared" si="6"/>
-        <v>prevalence_preclin_65</v>
+        <v>prevalence_preclin_85</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C12" s="1">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="D12" s="1">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="E12" s="1">
-        <f t="shared" si="0"/>
-        <v>65</v>
+        <f t="shared" si="1"/>
+        <v>85</v>
       </c>
       <c r="G12" s="1">
-        <v>1084</v>
+        <v>887</v>
       </c>
       <c r="H12" s="1">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="I12" s="1">
+        <f t="shared" si="2"/>
+        <v>2.5930101465614429E-2</v>
+      </c>
+      <c r="J12" s="1">
+        <f t="shared" si="3"/>
+        <v>4.330844217242529E-3</v>
+      </c>
+      <c r="K12" s="1">
+        <f t="shared" si="4"/>
+        <v>1.7339774526665963E-2</v>
+      </c>
+      <c r="L12" s="1">
         <f t="shared" si="5"/>
-        <v>1.5682656826568265E-2</v>
-      </c>
-      <c r="J12" s="1">
-        <f t="shared" si="1"/>
-        <v>3.543781199902328E-3</v>
-      </c>
-      <c r="K12" s="1">
-        <f t="shared" si="2"/>
-        <v>9.8142486381670446E-3</v>
-      </c>
-      <c r="L12" s="1">
-        <f t="shared" si="3"/>
-        <v>2.4971572874571808E-2</v>
+        <v>3.8608967336644713E-2</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="str">
         <f t="shared" si="6"/>
-        <v>prevalence_preclin_75</v>
+        <v>prevalence_preclin_95</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C13" s="1">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="D13" s="1">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="E13" s="1">
-        <f t="shared" si="0"/>
-        <v>75</v>
+        <f t="shared" si="1"/>
+        <v>95</v>
       </c>
       <c r="G13" s="1">
-        <v>1428</v>
+        <v>150</v>
       </c>
       <c r="H13" s="1">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="I13" s="1">
+        <f t="shared" si="2"/>
+        <v>1.3333333333333334E-2</v>
+      </c>
+      <c r="J13" s="1">
+        <f t="shared" si="3"/>
+        <v>2.5609725471294156E-2</v>
+      </c>
+      <c r="K13" s="1">
+        <f t="shared" si="4"/>
+        <v>3.6641291512270503E-3</v>
+      </c>
+      <c r="L13" s="1">
         <f t="shared" si="5"/>
-        <v>1.8207282913165267E-2</v>
-      </c>
-      <c r="J13" s="1">
-        <f t="shared" si="1"/>
-        <v>2.690097213371235E-3</v>
-      </c>
-      <c r="K13" s="1">
-        <f t="shared" si="2"/>
-        <v>1.2455064037696518E-2</v>
-      </c>
-      <c r="L13" s="1">
-        <f t="shared" si="3"/>
-        <v>2.6544685883420276E-2</v>
+        <v>4.7306908700367495E-2</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="str">
-        <f t="shared" si="6"/>
-        <v>prevalence_preclin_85</v>
+      <c r="A14" s="1" t="s">
+        <v>16</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" s="1">
-        <v>80</v>
-      </c>
-      <c r="D14" s="1">
-        <v>90</v>
+        <v>17</v>
       </c>
       <c r="E14" s="1">
-        <f t="shared" si="0"/>
-        <v>85</v>
+        <v>1</v>
       </c>
       <c r="G14" s="1">
-        <v>887</v>
+        <v>62758</v>
       </c>
       <c r="H14" s="1">
-        <v>23</v>
+        <v>11347</v>
       </c>
       <c r="I14" s="1">
-        <f t="shared" si="5"/>
-        <v>2.5930101465614429E-2</v>
+        <f t="shared" ref="I14:I17" si="7">H14/G14</f>
+        <v>0.18080563434143854</v>
       </c>
       <c r="J14" s="1">
-        <f t="shared" si="1"/>
-        <v>4.330844217242529E-3</v>
+        <f t="shared" ref="J14:J17" si="8">$B$4^2/G14</f>
+        <v>6.1210663512127909E-5</v>
       </c>
       <c r="K14" s="1">
-        <f t="shared" si="2"/>
-        <v>1.7339774526665963E-2</v>
+        <f t="shared" ref="K14:K17" si="9">(I14+J14/2)/(J14+1)-$B$4/(J14+1)*SQRT(I14*(1-I14)/G14+J14/(4*G14))</f>
+        <v>0.17781418443524724</v>
       </c>
       <c r="L14" s="1">
-        <f t="shared" si="3"/>
-        <v>3.8608967336644713E-2</v>
+        <f t="shared" ref="L14:L17" si="10">(I14+J14/2)/(J14+1)+$B$4/(J14+1)*SQRT(I14*(1-I14)/G14+J14/(4*G14))</f>
+        <v>0.18383615805371881</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="str">
-        <f t="shared" si="6"/>
-        <v>prevalence_preclin_95</v>
+      <c r="A15" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15" s="1">
-        <v>90</v>
-      </c>
-      <c r="D15" s="1">
-        <v>100</v>
+        <v>17</v>
       </c>
       <c r="E15" s="1">
-        <f t="shared" si="0"/>
-        <v>95</v>
+        <v>2</v>
       </c>
       <c r="G15" s="1">
-        <v>150</v>
+        <v>62758</v>
       </c>
       <c r="H15" s="1">
-        <v>2</v>
+        <v>21077</v>
       </c>
       <c r="I15" s="1">
-        <f t="shared" si="5"/>
-        <v>1.3333333333333334E-2</v>
+        <f t="shared" si="7"/>
+        <v>0.33584562924248701</v>
       </c>
       <c r="J15" s="1">
-        <f t="shared" si="1"/>
-        <v>2.5609725471294156E-2</v>
+        <f t="shared" si="8"/>
+        <v>6.1210663512127909E-5</v>
       </c>
       <c r="K15" s="1">
-        <f t="shared" si="2"/>
-        <v>3.6641291512270503E-3</v>
+        <f t="shared" si="9"/>
+        <v>0.33216074653492256</v>
       </c>
       <c r="L15" s="1">
-        <f t="shared" si="3"/>
-        <v>4.7306908700367495E-2</v>
+        <f t="shared" si="10"/>
+        <v>0.33955060671594262</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E16" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G16" s="1">
         <v>62758</v>
       </c>
       <c r="H16" s="1">
-        <v>11347</v>
+        <v>15405</v>
       </c>
       <c r="I16" s="1">
-        <f t="shared" ref="I16:I19" si="7">H16/G16</f>
-        <v>0.18080563434143854</v>
+        <f t="shared" si="7"/>
+        <v>0.24546671340705567</v>
       </c>
       <c r="J16" s="1">
-        <f t="shared" ref="J16:J19" si="8">$B$4^2/G16</f>
+        <f t="shared" si="8"/>
         <v>6.1210663512127909E-5</v>
       </c>
       <c r="K16" s="1">
-        <f t="shared" ref="K16:K19" si="9">(I16+J16/2)/(J16+1)-$B$4/(J16+1)*SQRT(I16*(1-I16)/G16+J16/(4*G16))</f>
-        <v>0.17781418443524724</v>
+        <f t="shared" si="9"/>
+        <v>0.24211531360934294</v>
       </c>
       <c r="L16" s="1">
-        <f t="shared" ref="L16:L19" si="10">(I16+J16/2)/(J16+1)+$B$4/(J16+1)*SQRT(I16*(1-I16)/G16+J16/(4*G16))</f>
-        <v>0.18383615805371881</v>
+        <f t="shared" si="10"/>
+        <v>0.24884927160025891</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E17" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G17" s="1">
         <v>62758</v>
       </c>
       <c r="H17" s="1">
-        <v>21077</v>
+        <v>14929</v>
       </c>
       <c r="I17" s="1">
         <f t="shared" si="7"/>
-        <v>0.33584562924248701</v>
+        <v>0.23788202300901878</v>
       </c>
       <c r="J17" s="1">
         <f t="shared" si="8"/>
@@ -2561,75 +2390,9 @@
       </c>
       <c r="K17" s="1">
         <f t="shared" si="9"/>
-        <v>0.33216074653492256</v>
+        <v>0.23456689332002215</v>
       </c>
       <c r="L17" s="1">
-        <f t="shared" si="10"/>
-        <v>0.33955060671594262</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E18" s="1">
-        <v>3</v>
-      </c>
-      <c r="G18" s="1">
-        <v>62758</v>
-      </c>
-      <c r="H18" s="1">
-        <v>15405</v>
-      </c>
-      <c r="I18" s="1">
-        <f t="shared" si="7"/>
-        <v>0.24546671340705567</v>
-      </c>
-      <c r="J18" s="1">
-        <f t="shared" si="8"/>
-        <v>6.1210663512127909E-5</v>
-      </c>
-      <c r="K18" s="1">
-        <f t="shared" si="9"/>
-        <v>0.24211531360934294</v>
-      </c>
-      <c r="L18" s="1">
-        <f t="shared" si="10"/>
-        <v>0.24884927160025891</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A19" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E19" s="1">
-        <v>4</v>
-      </c>
-      <c r="G19" s="1">
-        <v>62758</v>
-      </c>
-      <c r="H19" s="1">
-        <v>14929</v>
-      </c>
-      <c r="I19" s="1">
-        <f t="shared" si="7"/>
-        <v>0.23788202300901878</v>
-      </c>
-      <c r="J19" s="1">
-        <f t="shared" si="8"/>
-        <v>6.1210663512127909E-5</v>
-      </c>
-      <c r="K19" s="1">
-        <f t="shared" si="9"/>
-        <v>0.23456689332002215</v>
-      </c>
-      <c r="L19" s="1">
         <f t="shared" si="10"/>
         <v>0.24122923956453721</v>
       </c>

</xml_diff>